<commit_message>
Design updates in dataset files
</commit_message>
<xml_diff>
--- a/thesis/foundationalDataset/decision_dataset.xlsx
+++ b/thesis/foundationalDataset/decision_dataset.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oguzarslan/Desktop/Master Thesis Dataset/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/oguzarslan/Desktop/upc/semester-4/Thesis/MappingGenerator/thesis/foundationalDataset/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67BBC30E-41C9-6B4F-A06C-946AA817562C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22D01B5B-B903-424F-A425-29F8ABD6569A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4000" yWindow="1200" windowWidth="22080" windowHeight="16420" xr2:uid="{2B77A409-4A0A-9944-8DFB-55F0A25FF29E}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="276">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="376" uniqueCount="275">
   <si>
     <t>Document ID</t>
   </si>
@@ -619,12 +619,6 @@
     <t>*CF_M08_C10</t>
   </si>
   <si>
-    <t>Traefik opens port 80 to handle non-secure HTTP traffic re-</t>
-  </si>
-  <si>
-    <t>directing this traffic to port 443 (HTTPS) to ensure that all communications are carried out safely.</t>
-  </si>
-  <si>
     <t>CF_M08_AD03</t>
   </si>
   <si>
@@ -866,13 +860,16 @@
   </si>
   <si>
     <t>*CF_M08_C11, *CF_M08_C12, *CF_M08_C13</t>
+  </si>
+  <si>
+    <t>Traefik opens port 80 to handle non-secure HTTP traffic re-directing this traffic to port 443 (HTTPS) to ensure that all communications are carried out safely.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -890,26 +887,6 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color theme="0"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Arial"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -917,13 +894,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="9"/>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="12"/>
       <color rgb="FF000000"/>
-      <name val="Helvetica"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -938,13 +924,19 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFFFFF"/>
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFF6F8F9"/>
+        <fgColor theme="0"/>
         <bgColor rgb="FFF6F8F9"/>
       </patternFill>
     </fill>
@@ -961,39 +953,35 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="3" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="49" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1308,7 +1296,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{492A3DD4-FC69-984C-977C-946BA960D4E2}">
-  <dimension ref="A1:F76"/>
+  <dimension ref="A1:F75"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="15.6640625" customWidth="1"/>
@@ -1317,27 +1305,27 @@
     <col min="6" max="6" width="18.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" s="3" customFormat="1" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" s="1" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="F1" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" s="9" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="4" t="s">
         <v>6</v>
       </c>
@@ -1357,7 +1345,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="3" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="7" t="s">
         <v>6</v>
       </c>
@@ -1377,7 +1365,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="4" t="s">
         <v>6</v>
       </c>
@@ -1397,7 +1385,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="28" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="7" t="s">
         <v>6</v>
       </c>
@@ -1417,1424 +1405,1407 @@
         <v>46</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="51" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B6" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="C6" t="s">
+      <c r="C6" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="D6" t="s">
+      <c r="D6" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="9" t="s">
+      <c r="E6" s="10" t="s">
         <v>22</v>
       </c>
       <c r="F6" s="7">
         <v>46</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="68" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B7" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="D7" t="s">
+      <c r="D7" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E7" s="9" t="s">
+      <c r="E7" s="10" t="s">
         <v>26</v>
       </c>
       <c r="F7" s="7">
         <v>46</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C8" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D8" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="E8" t="s">
+      <c r="E8" s="9" t="s">
         <v>29</v>
       </c>
       <c r="F8" s="7">
         <v>50</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="7" t="s">
         <v>34</v>
       </c>
-      <c r="C9" t="s">
+      <c r="C9" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="D9" t="s">
+      <c r="D9" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="E9" t="s">
+      <c r="E9" s="9" t="s">
         <v>32</v>
       </c>
       <c r="F9" s="7">
         <v>49</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" t="s">
+    <row r="10" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A10" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C10" t="s">
+      <c r="C10" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D10" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="E10" t="s">
+      <c r="E10" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="9">
         <v>55</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" t="s">
+    <row r="11" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A11" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C11" t="s">
+      <c r="C11" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="D11" t="s">
+      <c r="D11" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="E11" t="s">
+      <c r="E11" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="F11">
+      <c r="F11" s="9">
         <v>56</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A12" t="s">
+    <row r="12" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A12" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B12" t="s">
+      <c r="B12" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C12" t="s">
+      <c r="C12" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="D12" t="s">
+      <c r="D12" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="E12" t="s">
+      <c r="E12" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="9">
         <v>56</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" t="s">
+    <row r="13" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A13" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B13" t="s">
+      <c r="B13" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="C13" t="s">
+      <c r="C13" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="D13" t="s">
+      <c r="D13" s="9" t="s">
         <v>50</v>
       </c>
-      <c r="E13" t="s">
+      <c r="E13" s="9" t="s">
         <v>51</v>
       </c>
-      <c r="F13">
+      <c r="F13" s="9">
         <v>62</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" t="s">
+    <row r="14" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A14" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="C14" t="s">
+      <c r="C14" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="D14" t="s">
+      <c r="D14" s="9" t="s">
         <v>54</v>
       </c>
-      <c r="E14" t="s">
+      <c r="E14" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="9">
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="102" x14ac:dyDescent="0.2">
-      <c r="A15" t="s">
+    <row r="15" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A15" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B15" t="s">
+      <c r="B15" s="9" t="s">
         <v>56</v>
       </c>
-      <c r="C15" t="s">
+      <c r="C15" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="D15" t="s">
+      <c r="D15" s="9" t="s">
         <v>57</v>
       </c>
-      <c r="E15" s="9" t="s">
+      <c r="E15" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="9">
         <v>64</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" t="s">
+    <row r="16" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A16" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B16" t="s">
+      <c r="B16" s="9" t="s">
         <v>59</v>
       </c>
-      <c r="C16" t="s">
+      <c r="C16" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D16" t="s">
+      <c r="D16" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E16" s="9" t="s">
         <v>62</v>
       </c>
-      <c r="F16">
+      <c r="F16" s="9">
         <v>64</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" t="s">
+    <row r="17" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A17" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B17" t="s">
+      <c r="B17" s="9" t="s">
         <v>63</v>
       </c>
-      <c r="C17" t="s">
+      <c r="C17" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="D17" t="s">
+      <c r="D17" s="9" t="s">
         <v>65</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E17" s="9" t="s">
         <v>66</v>
       </c>
-      <c r="F17">
+      <c r="F17" s="9">
         <v>67</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" t="s">
+    <row r="18" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A18" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B18" t="s">
+      <c r="B18" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="9" t="s">
         <v>68</v>
       </c>
-      <c r="D18" t="s">
+      <c r="D18" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E18" s="9" t="s">
         <v>69</v>
       </c>
-      <c r="F18">
+      <c r="F18" s="9">
         <v>68</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" t="s">
+    <row r="19" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A19" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B19" t="s">
+      <c r="B19" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D19" t="s">
+      <c r="D19" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E19" s="9" t="s">
         <v>72</v>
       </c>
-      <c r="F19">
+      <c r="F19" s="9">
         <v>70</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" t="s">
+    <row r="20" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A20" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B20" t="s">
+      <c r="B20" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D20" t="s">
+      <c r="D20" s="9" t="s">
         <v>74</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E20" s="9" t="s">
         <v>75</v>
       </c>
-      <c r="F20">
+      <c r="F20" s="9">
         <v>70</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" t="s">
+    <row r="21" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A21" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B21" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="9" t="s">
         <v>77</v>
       </c>
-      <c r="D21" t="s">
+      <c r="D21" s="9" t="s">
         <v>78</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E21" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="F21">
+      <c r="F21" s="9">
         <v>71</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" t="s">
+    <row r="22" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A22" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B22" t="s">
+      <c r="B22" s="9" t="s">
         <v>80</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="9" t="s">
         <v>60</v>
       </c>
-      <c r="D22" t="s">
+      <c r="D22" s="9" t="s">
         <v>81</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E22" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="F22">
+      <c r="F22" s="9">
         <v>72</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" t="s">
+    <row r="23" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A23" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B23" s="9" t="s">
         <v>83</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="D23" t="s">
+      <c r="D23" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E23" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="F23">
+      <c r="F23" s="9">
         <v>73</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" t="s">
+    <row r="24" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B24" t="s">
+      <c r="B24" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="C24" t="s">
+      <c r="C24" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="D24" t="s">
+      <c r="D24" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E24" s="9" t="s">
         <v>87</v>
       </c>
-      <c r="F24">
+      <c r="F24" s="9">
         <v>73</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" t="s">
+    <row r="25" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A25" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B25" t="s">
+      <c r="B25" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="C25" t="s">
+      <c r="C25" s="9" t="s">
         <v>89</v>
       </c>
-      <c r="D25" t="s">
+      <c r="D25" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E25" s="9" t="s">
         <v>90</v>
       </c>
-      <c r="F25">
+      <c r="F25" s="9">
         <v>73</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" t="s">
+    <row r="26" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A26" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B26" t="s">
+      <c r="B26" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="C26" t="s">
+      <c r="C26" s="9" t="s">
         <v>92</v>
       </c>
-      <c r="D26" t="s">
+      <c r="D26" s="9" t="s">
         <v>93</v>
       </c>
-      <c r="E26" t="s">
+      <c r="E26" s="9" t="s">
         <v>94</v>
       </c>
-      <c r="F26">
+      <c r="F26" s="9">
         <v>75</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" t="s">
+    <row r="27" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A27" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B27" t="s">
+      <c r="B27" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="C27" t="s">
+      <c r="C27" s="9" t="s">
         <v>53</v>
       </c>
-      <c r="D27" t="s">
+      <c r="D27" s="9" t="s">
         <v>96</v>
       </c>
-      <c r="E27" t="s">
+      <c r="E27" s="9" t="s">
         <v>97</v>
       </c>
-      <c r="F27">
+      <c r="F27" s="9">
         <v>84</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" t="s">
+    <row r="28" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A28" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B28" t="s">
+      <c r="B28" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="C28" t="s">
+      <c r="C28" s="9" t="s">
         <v>86</v>
       </c>
-      <c r="D28" t="s">
+      <c r="D28" s="9" t="s">
         <v>99</v>
       </c>
-      <c r="E28" t="s">
+      <c r="E28" s="9" t="s">
         <v>100</v>
       </c>
-      <c r="F28">
+      <c r="F28" s="9">
         <v>56</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" t="s">
+    <row r="29" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A29" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B29" t="s">
+      <c r="B29" s="9" t="s">
         <v>101</v>
       </c>
-      <c r="C29" t="s">
+      <c r="C29" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="D29" t="s">
+      <c r="D29" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="E29" t="s">
+      <c r="E29" s="9" t="s">
         <v>103</v>
       </c>
-      <c r="F29">
+      <c r="F29" s="9">
         <v>55</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" t="s">
+    <row r="30" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A30" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="B30" t="s">
+      <c r="B30" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="C30" t="s">
+      <c r="C30" s="9" t="s">
         <v>71</v>
       </c>
-      <c r="D30" t="s">
+      <c r="D30" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="E30" t="s">
+      <c r="E30" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="F30">
+      <c r="F30" s="9">
         <v>66</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A31" s="10" t="s">
+    <row r="31" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A31" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="C31" s="10" t="s">
+      <c r="C31" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="D31" s="10" t="s">
+      <c r="D31" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="E31" s="10" t="s">
+      <c r="E31" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="F31" s="10">
+      <c r="F31" s="9">
         <v>56</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32" s="10" t="s">
+    <row r="32" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A32" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="D32" s="10" t="s">
+      <c r="D32" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="E32" s="10" t="s">
+      <c r="E32" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="F32" s="10">
+      <c r="F32" s="9">
         <v>57</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A33" s="10" t="s">
+    <row r="33" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A33" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D33" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="E33" s="10" t="s">
+      <c r="E33" s="9" t="s">
         <v>119</v>
       </c>
-      <c r="F33" s="10">
+      <c r="F33" s="9">
         <v>57</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A34" s="10" t="s">
+    <row r="34" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A34" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="9" t="s">
         <v>120</v>
       </c>
-      <c r="C34" s="10" t="s">
+      <c r="C34" s="9" t="s">
         <v>121</v>
       </c>
-      <c r="D34" s="10" t="s">
+      <c r="D34" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="E34" s="10" t="s">
+      <c r="E34" s="9" t="s">
         <v>123</v>
       </c>
-      <c r="F34" s="10">
+      <c r="F34" s="9">
         <v>58</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="10" t="s">
+    <row r="35" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A35" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B35" s="10" t="s">
+      <c r="B35" s="9" t="s">
         <v>124</v>
       </c>
-      <c r="C35" s="10" t="s">
+      <c r="C35" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="D35" s="10" t="s">
+      <c r="D35" s="9" t="s">
         <v>126</v>
       </c>
-      <c r="E35" s="10" t="s">
+      <c r="E35" s="9" t="s">
         <v>127</v>
       </c>
-      <c r="F35" s="10">
+      <c r="F35" s="9">
         <v>58</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A36" s="10" t="s">
+    <row r="36" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A36" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B36" s="10" t="s">
+      <c r="B36" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="C36" s="9" t="s">
         <v>129</v>
       </c>
-      <c r="D36" s="10" t="s">
+      <c r="D36" s="9" t="s">
         <v>130</v>
       </c>
-      <c r="E36" s="10" t="s">
+      <c r="E36" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="F36" s="10">
+      <c r="F36" s="9">
         <v>60</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A37" s="10" t="s">
+    <row r="37" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A37" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B37" s="10" t="s">
+      <c r="B37" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="C37" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="D37" s="10" t="s">
+      <c r="D37" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="E37" s="10" t="s">
+      <c r="E37" s="9" t="s">
         <v>135</v>
       </c>
-      <c r="F37" s="10">
+      <c r="F37" s="9">
         <v>61</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A38" s="10" t="s">
+    <row r="38" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B38" s="10" t="s">
+      <c r="B38" s="9" t="s">
         <v>136</v>
       </c>
-      <c r="C38" s="10" t="s">
+      <c r="C38" s="9" t="s">
         <v>133</v>
       </c>
-      <c r="D38" s="10" t="s">
+      <c r="D38" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="E38" s="10" t="s">
+      <c r="E38" s="9" t="s">
         <v>138</v>
       </c>
-      <c r="F38" s="10">
+      <c r="F38" s="9">
         <v>61</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A39" s="10" t="s">
+    <row r="39" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B39" s="10" t="s">
+      <c r="B39" s="9" t="s">
         <v>139</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="D39" s="10" t="s">
+      <c r="D39" s="9" t="s">
         <v>141</v>
       </c>
-      <c r="E39" s="10" t="s">
+      <c r="E39" s="9" t="s">
         <v>142</v>
       </c>
-      <c r="F39" s="10">
+      <c r="F39" s="9">
         <v>76</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A40" s="10" t="s">
+    <row r="40" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A40" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B40" s="10" t="s">
+      <c r="B40" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="9" t="s">
         <v>144</v>
       </c>
-      <c r="D40" s="10" t="s">
+      <c r="D40" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="E40" s="10" t="s">
+      <c r="E40" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="F40" s="10">
+      <c r="F40" s="9">
         <v>77</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A41" s="10" t="s">
+    <row r="41" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A41" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B41" s="10" t="s">
+      <c r="B41" s="9" t="s">
         <v>147</v>
       </c>
-      <c r="C41" s="10" t="s">
+      <c r="C41" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="D41" s="10" t="s">
+      <c r="D41" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="E41" s="10" t="s">
+      <c r="E41" s="9" t="s">
         <v>150</v>
       </c>
-      <c r="F41" s="10">
+      <c r="F41" s="9">
         <v>81</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A42" s="10" t="s">
+    <row r="42" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A42" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B42" s="10" t="s">
+      <c r="B42" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="C42" s="11" t="s">
+      <c r="C42" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="D42" s="11" t="s">
+      <c r="D42" s="9" t="s">
         <v>145</v>
       </c>
-      <c r="E42" s="11" t="s">
+      <c r="E42" s="9" t="s">
         <v>153</v>
       </c>
-      <c r="F42" s="11">
+      <c r="F42" s="9">
         <v>78</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A43" s="10" t="s">
+    <row r="43" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A43" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="B43" s="10" t="s">
+      <c r="B43" s="9" t="s">
         <v>154</v>
       </c>
-      <c r="C43" s="11" t="s">
+      <c r="C43" s="9" t="s">
         <v>148</v>
       </c>
-      <c r="D43" s="11" t="s">
+      <c r="D43" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="E43" s="11" t="s">
+      <c r="E43" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="F43" s="11">
+      <c r="F43" s="9">
         <v>82</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A44" t="s">
+    <row r="44" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A44" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B44" t="s">
+      <c r="B44" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="C44" t="s">
+      <c r="C44" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="D44" t="s">
+      <c r="D44" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="E44" t="s">
+      <c r="E44" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="F44">
+      <c r="F44" s="9">
         <v>46</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A45" t="s">
+    <row r="45" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A45" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B45" t="s">
+      <c r="B45" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="C45" t="s">
+      <c r="C45" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="D45" t="s">
+      <c r="D45" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="E45" t="s">
+      <c r="E45" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="F45">
+      <c r="F45" s="9">
         <v>47</v>
       </c>
     </row>
-    <row r="46" spans="1:6" ht="85" x14ac:dyDescent="0.2">
-      <c r="A46" t="s">
+    <row r="46" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A46" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B46" t="s">
+      <c r="B46" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="C46" t="s">
+      <c r="C46" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="D46" t="s">
+      <c r="D46" s="9" t="s">
         <v>168</v>
       </c>
-      <c r="E46" s="9" t="s">
+      <c r="E46" s="10" t="s">
         <v>169</v>
       </c>
-      <c r="F46">
+      <c r="F46" s="9">
         <v>49</v>
       </c>
     </row>
-    <row r="47" spans="1:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="A47" t="s">
+    <row r="47" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A47" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B47" t="s">
+      <c r="B47" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="C47" t="s">
+      <c r="C47" s="9" t="s">
         <v>171</v>
       </c>
-      <c r="D47" t="s">
+      <c r="D47" s="9" t="s">
         <v>172</v>
       </c>
-      <c r="E47" s="9" t="s">
+      <c r="E47" s="10" t="s">
         <v>173</v>
       </c>
-      <c r="F47">
+      <c r="F47" s="9">
         <v>52</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A48" t="s">
+    <row r="48" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A48" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B48" t="s">
+      <c r="B48" s="9" t="s">
         <v>174</v>
       </c>
-      <c r="C48" t="s">
+      <c r="C48" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="D48" t="s">
+      <c r="D48" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="E48" t="s">
+      <c r="E48" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="F48">
+      <c r="F48" s="9">
         <v>51</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A49" t="s">
+    <row r="49" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A49" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B49" t="s">
+      <c r="B49" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="C49" t="s">
+      <c r="C49" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="D49" t="s">
+      <c r="D49" s="9" t="s">
         <v>175</v>
       </c>
-      <c r="E49" s="12" t="s">
+      <c r="E49" s="11" t="s">
         <v>178</v>
       </c>
-      <c r="F49">
+      <c r="F49" s="9">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A50" t="s">
+    <row r="50" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A50" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B50" t="s">
+      <c r="B50" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="C50" t="s">
+      <c r="C50" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="D50" t="s">
+      <c r="D50" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="E50" t="s">
+      <c r="E50" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="F50">
+      <c r="F50" s="9">
         <v>92</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A51" t="s">
+    <row r="51" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A51" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="B51" t="s">
+      <c r="B51" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="C51" t="s">
+      <c r="C51" s="9" t="s">
         <v>180</v>
       </c>
-      <c r="D51" t="s">
+      <c r="D51" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="E51" t="s">
+      <c r="E51" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="F51">
+      <c r="F51" s="9">
         <v>92</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A52" s="13" t="s">
+    <row r="52" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A52" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B52" s="13" t="s">
+      <c r="B52" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="C52" s="13" t="s">
+      <c r="C52" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="D52" s="13" t="s">
+      <c r="D52" s="9" t="s">
         <v>189</v>
       </c>
-      <c r="E52" s="13" t="s">
+      <c r="E52" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="F52" s="13">
+      <c r="F52" s="9">
         <v>43</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A53" s="14" t="s">
+    <row r="53" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A53" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B53" s="15" t="s">
+      <c r="B53" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="C53" s="14" t="s">
+      <c r="C53" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="D53" s="15" t="s">
+      <c r="D53" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="E53" s="13" t="s">
+      <c r="E53" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="F53" s="9">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A54" s="9" t="s">
+        <v>186</v>
+      </c>
+      <c r="B54" s="9" t="s">
         <v>193</v>
       </c>
-      <c r="F53" s="15">
+      <c r="C54" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="D54" s="9" t="s">
+        <v>273</v>
+      </c>
+      <c r="E54" s="9" t="s">
+        <v>195</v>
+      </c>
+      <c r="F54" s="9">
         <v>43</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A54" s="14"/>
-      <c r="B54" s="15"/>
-      <c r="C54" s="14"/>
-      <c r="D54" s="15"/>
-      <c r="E54" s="13" t="s">
-        <v>194</v>
-      </c>
-      <c r="F54" s="15"/>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A55" s="13" t="s">
+    <row r="55" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A55" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B55" s="10" t="s">
-        <v>195</v>
-      </c>
-      <c r="C55" s="13" t="s">
+      <c r="B55" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="D55" s="10" t="s">
-        <v>275</v>
-      </c>
-      <c r="E55" s="13" t="s">
+      <c r="C55" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="F55" s="10">
-        <v>43</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A56" s="13" t="s">
+      <c r="D55" s="9" t="s">
+        <v>198</v>
+      </c>
+      <c r="E55" s="9" t="s">
+        <v>199</v>
+      </c>
+      <c r="F55" s="9">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A56" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B56" s="10" t="s">
-        <v>198</v>
-      </c>
-      <c r="C56" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="D56" s="10" t="s">
+      <c r="B56" s="9" t="s">
         <v>200</v>
       </c>
-      <c r="E56" s="13" t="s">
+      <c r="C56" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="D56" s="9" t="s">
         <v>201</v>
       </c>
-      <c r="F56" s="10">
+      <c r="E56" s="9" t="s">
+        <v>202</v>
+      </c>
+      <c r="F56" s="9">
         <v>45</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A57" s="13" t="s">
+    <row r="57" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A57" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B57" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="C57" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="D57" s="10" t="s">
+      <c r="B57" s="9" t="s">
         <v>203</v>
       </c>
-      <c r="E57" s="13" t="s">
+      <c r="C57" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="D57" s="9" t="s">
         <v>204</v>
       </c>
-      <c r="F57" s="10">
+      <c r="E57" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="F57" s="9">
         <v>45</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A58" s="13" t="s">
+    <row r="58" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A58" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B58" s="10" t="s">
-        <v>205</v>
-      </c>
-      <c r="C58" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="D58" s="10" t="s">
+      <c r="B58" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="E58" s="13" t="s">
+      <c r="C58" s="9" t="s">
+        <v>197</v>
+      </c>
+      <c r="D58" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="F58" s="10">
-        <v>45</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A59" s="13" t="s">
+      <c r="E58" s="9" t="s">
+        <v>208</v>
+      </c>
+      <c r="F58" s="9">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A59" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B59" s="10" t="s">
-        <v>208</v>
-      </c>
-      <c r="C59" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="D59" s="10" t="s">
+      <c r="B59" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="E59" s="13" t="s">
+      <c r="C59" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="F59" s="10">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A60" s="13" t="s">
+      <c r="D59" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="E59" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="F59" s="9">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A60" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B60" s="10" t="s">
-        <v>211</v>
-      </c>
-      <c r="C60" s="13" t="s">
-        <v>212</v>
-      </c>
-      <c r="D60" s="10" t="s">
+      <c r="B60" s="9" t="s">
         <v>213</v>
       </c>
-      <c r="E60" s="13" t="s">
+      <c r="C60" s="9" t="s">
+        <v>210</v>
+      </c>
+      <c r="D60" s="9" t="s">
         <v>214</v>
       </c>
-      <c r="F60" s="10">
+      <c r="E60" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="F60" s="9">
         <v>47</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A61" s="13" t="s">
+    <row r="61" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A61" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B61" s="10" t="s">
-        <v>215</v>
-      </c>
-      <c r="C61" s="13" t="s">
-        <v>212</v>
-      </c>
-      <c r="D61" s="10" t="s">
+      <c r="B61" s="9" t="s">
         <v>216</v>
       </c>
-      <c r="E61" s="13" t="s">
+      <c r="C61" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="F61" s="10">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A62" s="13" t="s">
+      <c r="D61" s="9" t="s">
+        <v>218</v>
+      </c>
+      <c r="E61" s="9" t="s">
+        <v>219</v>
+      </c>
+      <c r="F61" s="9">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A62" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B62" s="10" t="s">
-        <v>218</v>
-      </c>
-      <c r="C62" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="D62" s="10" t="s">
+      <c r="B62" s="9" t="s">
         <v>220</v>
       </c>
-      <c r="E62" s="13" t="s">
+      <c r="C62" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="D62" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="F62" s="10">
+      <c r="E62" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="F62" s="9">
         <v>50</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A63" s="13" t="s">
+    <row r="63" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A63" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B63" s="10" t="s">
-        <v>222</v>
-      </c>
-      <c r="C63" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="D63" s="10" t="s">
+      <c r="B63" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="E63" s="13" t="s">
+      <c r="C63" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="D63" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="F63" s="10">
+      <c r="E63" s="9" t="s">
+        <v>225</v>
+      </c>
+      <c r="F63" s="9">
         <v>50</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A64" s="13" t="s">
+    <row r="64" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A64" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B64" s="10" t="s">
-        <v>225</v>
-      </c>
-      <c r="C64" s="13" t="s">
-        <v>219</v>
-      </c>
-      <c r="D64" s="10" t="s">
+      <c r="B64" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="E64" s="13" t="s">
+      <c r="C64" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="F64" s="10">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A65" s="13" t="s">
+      <c r="D64" s="9" t="s">
+        <v>228</v>
+      </c>
+      <c r="E64" s="9" t="s">
+        <v>229</v>
+      </c>
+      <c r="F64" s="9">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A65" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="B65" s="10" t="s">
-        <v>228</v>
-      </c>
-      <c r="C65" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="D65" s="10" t="s">
+      <c r="B65" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="E65" s="13" t="s">
+      <c r="C65" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="F65" s="10">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A66" s="13" t="s">
-        <v>186</v>
-      </c>
-      <c r="B66" s="10" t="s">
+      <c r="D65" s="9" t="s">
         <v>232</v>
       </c>
-      <c r="C66" s="13" t="s">
+      <c r="E65" s="9" t="s">
         <v>233</v>
       </c>
-      <c r="D66" s="10" t="s">
+      <c r="F65" s="9">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A66" s="9" t="s">
         <v>234</v>
       </c>
-      <c r="E66" s="13" t="s">
+      <c r="B66" s="9" t="s">
         <v>235</v>
       </c>
-      <c r="F66" s="10">
-        <v>66</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A67" s="11" t="s">
+      <c r="C66" s="9" t="s">
         <v>236</v>
       </c>
-      <c r="B67" s="11" t="s">
+      <c r="D66" s="9" t="s">
         <v>237</v>
       </c>
-      <c r="C67" s="11" t="s">
+      <c r="E66" s="9" t="s">
         <v>238</v>
       </c>
-      <c r="D67" s="11" t="s">
+      <c r="F66" s="9">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A67" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B67" s="9" t="s">
         <v>239</v>
       </c>
-      <c r="E67" s="11" t="s">
+      <c r="C67" s="9" t="s">
         <v>240</v>
       </c>
-      <c r="F67" s="11">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A68" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="B68" s="11" t="s">
+      <c r="D67" s="9" t="s">
         <v>241</v>
       </c>
-      <c r="C68" s="11" t="s">
+      <c r="E67" s="9" t="s">
         <v>242</v>
       </c>
-      <c r="D68" s="11" t="s">
+      <c r="F67" s="9">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A68" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B68" s="9" t="s">
         <v>243</v>
       </c>
-      <c r="E68" s="11" t="s">
+      <c r="C68" s="9" t="s">
         <v>244</v>
       </c>
-      <c r="F68" s="11">
+      <c r="D68" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="E68" s="9" t="s">
+        <v>246</v>
+      </c>
+      <c r="F68" s="9">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A69" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B69" s="9" t="s">
+        <v>247</v>
+      </c>
+      <c r="C69" s="9" t="s">
+        <v>248</v>
+      </c>
+      <c r="D69" s="9" t="s">
+        <v>249</v>
+      </c>
+      <c r="E69" s="9" t="s">
+        <v>250</v>
+      </c>
+      <c r="F69" s="9">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A70" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B70" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="C70" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>253</v>
+      </c>
+      <c r="E70" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="F70" s="9">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A71" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B71" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="C71" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="D71" s="9" t="s">
+        <v>257</v>
+      </c>
+      <c r="E71" s="9" t="s">
+        <v>258</v>
+      </c>
+      <c r="F71" s="9">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A72" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B72" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="C72" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="D72" s="9" t="s">
+        <v>241</v>
+      </c>
+      <c r="E72" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="F72" s="9">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A73" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B73" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="C73" s="9" t="s">
+        <v>244</v>
+      </c>
+      <c r="D73" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="E73" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="F73" s="9">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A74" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B74" s="9" t="s">
+        <v>265</v>
+      </c>
+      <c r="C74" s="9" t="s">
+        <v>266</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>267</v>
+      </c>
+      <c r="E74" s="9" t="s">
+        <v>268</v>
+      </c>
+      <c r="F74" s="9">
         <v>57</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A69" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="B69" s="11" t="s">
-        <v>245</v>
-      </c>
-      <c r="C69" s="11" t="s">
-        <v>246</v>
-      </c>
-      <c r="D69" s="11" t="s">
-        <v>247</v>
-      </c>
-      <c r="E69" s="11" t="s">
-        <v>248</v>
-      </c>
-      <c r="F69" s="11">
+    <row r="75" spans="1:6" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A75" s="9" t="s">
+        <v>234</v>
+      </c>
+      <c r="B75" s="9" t="s">
+        <v>269</v>
+      </c>
+      <c r="C75" s="9" t="s">
+        <v>270</v>
+      </c>
+      <c r="D75" s="9" t="s">
+        <v>271</v>
+      </c>
+      <c r="E75" s="9" t="s">
+        <v>272</v>
+      </c>
+      <c r="F75" s="9">
         <v>58</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A70" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="B70" s="11" t="s">
-        <v>249</v>
-      </c>
-      <c r="C70" s="11" t="s">
-        <v>250</v>
-      </c>
-      <c r="D70" s="11" t="s">
-        <v>251</v>
-      </c>
-      <c r="E70" s="11" t="s">
-        <v>252</v>
-      </c>
-      <c r="F70" s="11">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A71" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="B71" s="11" t="s">
-        <v>253</v>
-      </c>
-      <c r="C71" s="11" t="s">
-        <v>254</v>
-      </c>
-      <c r="D71" s="11" t="s">
-        <v>255</v>
-      </c>
-      <c r="E71" s="11" t="s">
-        <v>256</v>
-      </c>
-      <c r="F71" s="11">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A72" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="B72" s="11" t="s">
-        <v>257</v>
-      </c>
-      <c r="C72" s="11" t="s">
-        <v>258</v>
-      </c>
-      <c r="D72" s="11" t="s">
-        <v>259</v>
-      </c>
-      <c r="E72" s="11" t="s">
-        <v>260</v>
-      </c>
-      <c r="F72" s="11">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A73" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="B73" s="11" t="s">
-        <v>261</v>
-      </c>
-      <c r="C73" s="11" t="s">
-        <v>262</v>
-      </c>
-      <c r="D73" s="11" t="s">
-        <v>243</v>
-      </c>
-      <c r="E73" s="11" t="s">
-        <v>263</v>
-      </c>
-      <c r="F73" s="11">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A74" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="B74" s="11" t="s">
-        <v>264</v>
-      </c>
-      <c r="C74" s="11" t="s">
-        <v>246</v>
-      </c>
-      <c r="D74" s="11" t="s">
-        <v>265</v>
-      </c>
-      <c r="E74" s="11" t="s">
-        <v>266</v>
-      </c>
-      <c r="F74" s="11">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A75" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="B75" s="11" t="s">
-        <v>267</v>
-      </c>
-      <c r="C75" s="11" t="s">
-        <v>268</v>
-      </c>
-      <c r="D75" s="11" t="s">
-        <v>269</v>
-      </c>
-      <c r="E75" s="11" t="s">
-        <v>270</v>
-      </c>
-      <c r="F75" s="11">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A76" s="11" t="s">
-        <v>236</v>
-      </c>
-      <c r="B76" s="11" t="s">
-        <v>271</v>
-      </c>
-      <c r="C76" s="11" t="s">
-        <v>272</v>
-      </c>
-      <c r="D76" s="11" t="s">
-        <v>273</v>
-      </c>
-      <c r="E76" s="11" t="s">
-        <v>274</v>
-      </c>
-      <c r="F76" s="11">
-        <v>58</v>
-      </c>
-    </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A53:A54"/>
-    <mergeCell ref="B53:B54"/>
-    <mergeCell ref="C53:C54"/>
-    <mergeCell ref="D53:D54"/>
-    <mergeCell ref="F53:F54"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>